<commit_message>
feat: add notification system, cleanup migrations, update README
</commit_message>
<xml_diff>
--- a/public/template/pelanggan.xlsx
+++ b/public/template/pelanggan.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ajes9\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\Aplikasi-Sistem-Manajemen-Tagihan-Pembayaran-Internet\public\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA536798-1B70-4321-8F4E-EA66966D8689}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C96F61F-339B-4A6D-964E-3BA96A76F67F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="15">
   <si>
     <t>Desa Pamutih</t>
   </si>
@@ -34,9 +34,6 @@
     <t>cst64@mail.com</t>
   </si>
   <si>
-    <t>Tanggal 11</t>
-  </si>
-  <si>
     <t>P004</t>
   </si>
   <si>
@@ -61,9 +58,6 @@
     <t>status</t>
   </si>
   <si>
-    <t>jatuh_tempo</t>
-  </si>
-  <si>
     <t>tanggal_pasang</t>
   </si>
   <si>
@@ -71,9 +65,6 @@
   </si>
   <si>
     <t>cst65@mail.com</t>
-  </si>
-  <si>
-    <t>Tanggal 20</t>
   </si>
 </sst>
 </file>
@@ -81,7 +72,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="169" formatCode="yyyy\-mm\-dd;@"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -128,7 +119,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
@@ -436,7 +427,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.21875" bestFit="1" customWidth="1"/>
@@ -446,40 +437,36 @@
     <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="7.88671875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="7.77734375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.21875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" t="s">
         <v>6</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>8</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>9</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>10</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>11</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>12</v>
       </c>
-      <c r="H1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I1" t="s">
-        <v>14</v>
-      </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -496,21 +483,18 @@
         <v>12345678</v>
       </c>
       <c r="F2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G2" t="s">
         <v>1</v>
       </c>
-      <c r="H2" t="s">
-        <v>4</v>
-      </c>
-      <c r="I2" s="3">
+      <c r="H2" s="3">
         <v>45791</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B3" t="s">
         <v>0</v>
@@ -519,25 +503,22 @@
         <v>6289673219746</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E3">
         <v>12345678</v>
       </c>
       <c r="F3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G3" t="s">
         <v>1</v>
       </c>
-      <c r="H3" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="I3" s="3">
+      <c r="H3" s="3">
         <v>45792</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C7" s="1"/>
     </row>
   </sheetData>

</xml_diff>